<commit_message>
Code setup to start co-writing the feature engineering code
Saves a sample of the data for testing, also updates the EDS script so that it saves "FirstCutData.rds" as the results of the merging work done in that script.

Also contains a new script called Preprocessing.R which we will work on together to write the feature preprocessing code
</commit_message>
<xml_diff>
--- a/Data/FieldActions.xlsx
+++ b/Data/FieldActions.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10727"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/raychandonnet/Chandonnet Family Dropbox/Chandonnet Family Folder/Ray Personal Stuff/Merrimack_MSDS/Capstone/MSDS-capstone/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16CF1E1C-F8FB-8440-A209-7FEF9222634A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6E1D5D2-94B5-354C-A22A-FBCC71FC49AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38400" yWindow="640" windowWidth="33500" windowHeight="20800" xr2:uid="{5D7287F0-0A17-C64B-9A67-8B848C646587}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="FieldActions" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">FieldActions!$A$1:$F$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">FieldActions!$A$1:$F$62</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="164">
   <si>
     <t>Homicides</t>
   </si>
@@ -278,18 +278,12 @@
     <t>PV.EST</t>
   </si>
   <si>
-    <t>GNIPerCap</t>
-  </si>
-  <si>
     <t>GNI per capita (annual % growth)</t>
   </si>
   <si>
     <t>NY.GNP.PCAP.KD.ZG</t>
   </si>
   <si>
-    <t>GDPPerCap</t>
-  </si>
-  <si>
     <t>GDP per capita (annual % growth)</t>
   </si>
   <si>
@@ -513,6 +507,30 @@
   </si>
   <si>
     <t>Predictor</t>
+  </si>
+  <si>
+    <t>NY.GDP.MKTP.KD.ZG</t>
+  </si>
+  <si>
+    <t>NY.GDP.MKTP.KD</t>
+  </si>
+  <si>
+    <t>GDP in USD</t>
+  </si>
+  <si>
+    <t>GDP in USD (annual % growth)</t>
+  </si>
+  <si>
+    <t>GDPPerCapGrowth</t>
+  </si>
+  <si>
+    <t>GNIPerCapGrowth</t>
+  </si>
+  <si>
+    <t>GDPGrowth</t>
+  </si>
+  <si>
+    <t>GDP</t>
   </si>
 </sst>
 </file>
@@ -872,7 +890,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41FC704B-350A-5F48-B132-84830513F75F}">
-  <dimension ref="A1:F60"/>
+  <dimension ref="A1:F62"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="48.5" bestFit="1" customWidth="1"/>
@@ -883,27 +901,27 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B2" t="s">
         <v>23</v>
@@ -914,63 +932,63 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B3" t="s">
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="E3" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B4" t="s">
         <v>2</v>
       </c>
       <c r="D4" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="E4" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B5" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="D5" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="E5" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B6" t="s">
         <v>2</v>
       </c>
       <c r="D6" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="E6" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B7" t="s">
         <v>23</v>
@@ -981,7 +999,7 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B8" t="s">
         <v>23</v>
@@ -992,35 +1010,35 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B9" t="s">
         <v>2</v>
       </c>
       <c r="D9" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="E9" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B10" t="s">
         <v>2</v>
       </c>
       <c r="D10" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="E10" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B11" t="s">
         <v>23</v>
@@ -1029,12 +1047,12 @@
         <v>#N/A</v>
       </c>
       <c r="F11" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B12" t="s">
         <v>23</v>
@@ -1043,12 +1061,12 @@
         <v>#N/A</v>
       </c>
       <c r="F12" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="B13" t="s">
         <v>23</v>
@@ -1057,12 +1075,12 @@
         <v>#N/A</v>
       </c>
       <c r="F13" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="3" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B14" t="s">
         <v>23</v>
@@ -1071,12 +1089,12 @@
         <v>#N/A</v>
       </c>
       <c r="F14" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B15" t="s">
         <v>23</v>
@@ -1085,12 +1103,12 @@
         <v>#N/A</v>
       </c>
       <c r="F15" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B16" t="s">
         <v>23</v>
@@ -1099,12 +1117,12 @@
         <v>#N/A</v>
       </c>
       <c r="F16" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" s="3" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B17" t="s">
         <v>23</v>
@@ -1113,12 +1131,12 @@
         <v>#N/A</v>
       </c>
       <c r="F17" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" s="3" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B18" t="s">
         <v>23</v>
@@ -1127,12 +1145,12 @@
         <v>#N/A</v>
       </c>
       <c r="F18" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" s="3" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B19" t="s">
         <v>23</v>
@@ -1141,12 +1159,12 @@
         <v>#N/A</v>
       </c>
       <c r="F19" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" s="3" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="B20" t="s">
         <v>23</v>
@@ -1155,12 +1173,12 @@
         <v>#N/A</v>
       </c>
       <c r="F20" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" s="3" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B21" t="s">
         <v>23</v>
@@ -1169,242 +1187,242 @@
         <v>#N/A</v>
       </c>
       <c r="F21" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" s="3" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B22" t="s">
         <v>2</v>
       </c>
       <c r="C22" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D22" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="E22" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" s="3" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B23" t="s">
         <v>2</v>
       </c>
       <c r="C23" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D23" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="E23" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" s="3" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B24" t="s">
         <v>2</v>
       </c>
       <c r="C24" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="D24" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E24" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" s="3" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B25" t="s">
         <v>2</v>
       </c>
       <c r="C25" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="D25" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="E25" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" s="3" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B26" t="s">
         <v>2</v>
       </c>
       <c r="C26" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D26" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="E26" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" s="3" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B27" t="s">
         <v>2</v>
       </c>
       <c r="C27" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D27" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="E27" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" s="3" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B28" t="s">
         <v>2</v>
       </c>
       <c r="C28" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D28" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="E28" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29" s="3" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B29" t="s">
         <v>2</v>
       </c>
       <c r="C29" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D29" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="E29" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30" s="3" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B30" t="s">
         <v>2</v>
       </c>
       <c r="C30" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D30" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E30" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31" s="3" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B31" t="s">
         <v>2</v>
       </c>
       <c r="C31" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="D31" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E31" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A32" s="3" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B32" t="s">
         <v>2</v>
       </c>
       <c r="C32" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D32" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="E32" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A33" s="3" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B33" t="s">
         <v>2</v>
       </c>
       <c r="C33" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="D33" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="E33" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A34" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B34" t="s">
         <v>2</v>
       </c>
       <c r="C34" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D34" t="s">
-        <v>82</v>
+        <v>160</v>
       </c>
       <c r="E34" t="s">
-        <v>10</v>
+        <v>155</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B35" t="s">
         <v>2</v>
       </c>
       <c r="C35" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D35" t="s">
-        <v>79</v>
+        <v>161</v>
       </c>
       <c r="E35" t="s">
         <v>10</v>
@@ -1412,84 +1430,84 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36" s="3" t="s">
-        <v>78</v>
+        <v>156</v>
       </c>
       <c r="B36" t="s">
         <v>2</v>
       </c>
       <c r="C36" t="s">
-        <v>77</v>
+        <v>159</v>
       </c>
       <c r="D36" t="s">
-        <v>76</v>
+        <v>162</v>
       </c>
       <c r="E36" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A37" s="3" t="s">
-        <v>75</v>
+        <v>157</v>
       </c>
       <c r="B37" t="s">
         <v>2</v>
       </c>
       <c r="C37" t="s">
-        <v>74</v>
+        <v>158</v>
       </c>
       <c r="D37" t="s">
-        <v>73</v>
+        <v>163</v>
       </c>
       <c r="E37" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A38" s="3" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="B38" t="s">
         <v>2</v>
       </c>
       <c r="C38" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="D38" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="E38" t="s">
-        <v>10</v>
+        <v>155</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A39" s="3" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="B39" t="s">
         <v>2</v>
       </c>
       <c r="C39" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="D39" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="E39" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A40" s="3" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="B40" t="s">
         <v>2</v>
       </c>
       <c r="C40" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="D40" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="E40" t="s">
         <v>10</v>
@@ -1497,33 +1515,33 @@
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A41" s="3" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="B41" t="s">
         <v>2</v>
       </c>
       <c r="C41" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="D41" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="E41" t="s">
-        <v>10</v>
+        <v>155</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A42" s="3" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="B42" t="s">
         <v>2</v>
       </c>
       <c r="C42" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="D42" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="E42" t="s">
         <v>10</v>
@@ -1531,16 +1549,16 @@
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A43" s="3" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="B43" t="s">
         <v>2</v>
       </c>
       <c r="C43" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="D43" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="E43" t="s">
         <v>10</v>
@@ -1548,16 +1566,16 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A44" s="3" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="B44" t="s">
         <v>2</v>
       </c>
       <c r="C44" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="D44" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="E44" t="s">
         <v>10</v>
@@ -1565,16 +1583,16 @@
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A45" s="3" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="B45" t="s">
         <v>2</v>
       </c>
       <c r="C45" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="D45" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="E45" t="s">
         <v>10</v>
@@ -1582,16 +1600,16 @@
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A46" s="3" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="B46" t="s">
         <v>2</v>
       </c>
       <c r="C46" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="D46" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="E46" t="s">
         <v>10</v>
@@ -1599,16 +1617,16 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A47" s="3" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="B47" t="s">
         <v>2</v>
       </c>
       <c r="C47" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="D47" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="E47" t="s">
         <v>10</v>
@@ -1616,16 +1634,16 @@
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A48" s="3" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="B48" t="s">
         <v>2</v>
       </c>
       <c r="C48" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="D48" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="E48" t="s">
         <v>10</v>
@@ -1633,213 +1651,247 @@
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A49" s="3" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="B49" t="s">
         <v>2</v>
       </c>
       <c r="C49" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="D49" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="E49" t="s">
-        <v>157</v>
+        <v>10</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A50" s="3" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="B50" t="s">
         <v>2</v>
       </c>
       <c r="C50" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D50" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="E50" t="s">
-        <v>157</v>
+        <v>10</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A51" s="3" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="B51" t="s">
         <v>2</v>
       </c>
       <c r="C51" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="D51" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="E51" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A52" s="3" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="B52" t="s">
         <v>2</v>
       </c>
       <c r="C52" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="D52" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="E52" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A53" s="3" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="B53" t="s">
         <v>2</v>
       </c>
       <c r="C53" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="D53" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="E53" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A54" s="3" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="B54" t="s">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="C54" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="D54" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="E54" t="s">
-        <v>10</v>
-      </c>
-      <c r="F54" t="s">
-        <v>20</v>
+        <v>155</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A55" s="3" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="B55" t="s">
         <v>2</v>
       </c>
       <c r="C55" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="D55" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="E55" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A56" s="3" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="B56" t="s">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="C56" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="D56" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="E56" t="s">
-        <v>157</v>
+        <v>10</v>
+      </c>
+      <c r="F56" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A57" s="3" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="B57" t="s">
         <v>2</v>
       </c>
       <c r="C57" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="D57" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="E57" t="s">
-        <v>10</v>
+        <v>155</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A58" s="3" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="B58" t="s">
         <v>2</v>
       </c>
       <c r="C58" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="D58" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="E58" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A59" s="3" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="B59" t="s">
         <v>2</v>
       </c>
       <c r="C59" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D59" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="E59" t="s">
-        <v>157</v>
+        <v>10</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A60" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B60" t="s">
+        <v>2</v>
+      </c>
+      <c r="C60" t="s">
+        <v>8</v>
+      </c>
+      <c r="D60" t="s">
+        <v>7</v>
+      </c>
+      <c r="E60" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A61" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B61" t="s">
+        <v>2</v>
+      </c>
+      <c r="C61" t="s">
+        <v>5</v>
+      </c>
+      <c r="D61" t="s">
+        <v>4</v>
+      </c>
+      <c r="E61" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A62" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B60" t="s">
-        <v>2</v>
-      </c>
-      <c r="C60" t="s">
+      <c r="B62" t="s">
+        <v>2</v>
+      </c>
+      <c r="C62" t="s">
         <v>1</v>
       </c>
-      <c r="D60" t="s">
+      <c r="D62" t="s">
         <v>0</v>
       </c>
-      <c r="E60" t="s">
-        <v>157</v>
+      <c r="E62" t="s">
+        <v>155</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F60" xr:uid="{41FC704B-350A-5F48-B132-84830513F75F}"/>
+  <autoFilter ref="A1:F62" xr:uid="{41FC704B-350A-5F48-B132-84830513F75F}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>